<commit_message>
Regenerate results json and xlsx with the new columns and provenance (existing values identical)
The json, xlsx and summary files of all 8 images come from a fresh default
run (every switch off). The golden test showed every existing field, cell
and column identical; the files gain the appended columns, the provenance
block and image_label. The PNG files were identical and are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/542_z06/2_canaliculi/542_z06_canaliculi_results.xlsx
+++ b/results/542_z06/2_canaliculi/542_z06_canaliculi_results.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -682,6 +682,441 @@
         </is>
       </c>
       <c r="G11" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>perimeter_px</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>normalised</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>297.8123</v>
+      </c>
+      <c r="D12" t="n">
+        <v>309.5219</v>
+      </c>
+      <c r="E12" t="n">
+        <v>115.1171</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>px</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ring_area_r30_px2</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>normalised</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>10771.6923</v>
+      </c>
+      <c r="D13" t="n">
+        <v>11337</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2967.4305</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>px^2</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ring_area_r60_px2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>normalised</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>25565.4615</v>
+      </c>
+      <c r="D14" t="n">
+        <v>27170</v>
+      </c>
+      <c r="E14" t="n">
+        <v>6351.0485</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>px^2</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>in_frame_fraction_r30</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>normalised</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>unitless</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>in_frame_fraction_r60</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>normalised</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.9908</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.0272</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>unitless</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ring_density_r30</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>normalised</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.03275532</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.03378319</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.00638738</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>px^-1</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ring_density_r60</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>normalised</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.0350223</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.03388488</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.00605335</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>px^-1</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>roots_per_100px_perimeter</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>normalised</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2.9437</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3.0734</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.4703</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>per 100 px</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ring_attached_length_r30_px</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>network v2</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>273.3077</v>
+      </c>
+      <c r="D20" t="n">
+        <v>276</v>
+      </c>
+      <c r="E20" t="n">
+        <v>139.0787</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>px</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ring_attached_length_r60_px</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>network v2</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>501</v>
+      </c>
+      <c r="D21" t="n">
+        <v>371</v>
+      </c>
+      <c r="E21" t="n">
+        <v>292.6622</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>px</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ring_length_w_r30_px</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>network v2</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>408.2629</v>
+      </c>
+      <c r="D22" t="n">
+        <v>353.8061</v>
+      </c>
+      <c r="E22" t="n">
+        <v>174.9104</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>px</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ring_length_w_r60_px</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>network v2</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1023.9562</v>
+      </c>
+      <c r="D23" t="n">
+        <v>920.193</v>
+      </c>
+      <c r="E23" t="n">
+        <v>381.4612</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>px</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>sholl_crossings_r10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>network v2</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>9.7692</v>
+      </c>
+      <c r="D24" t="n">
+        <v>10</v>
+      </c>
+      <c r="E24" t="n">
+        <v>4.5854</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>sholl_crossings_r20</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>network v2</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>12.5385</v>
+      </c>
+      <c r="D25" t="n">
+        <v>11</v>
+      </c>
+      <c r="E25" t="n">
+        <v>5.1416</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>sholl_crossings_r30</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>network v2</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>14</v>
+      </c>
+      <c r="D26" t="n">
+        <v>15</v>
+      </c>
+      <c r="E26" t="n">
+        <v>5.6421</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
         <v>13</v>
       </c>
     </row>
@@ -696,7 +1131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -918,6 +1353,63 @@
       <c r="D11" t="inlineStr">
         <is>
           <t>px</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>field_length_density_w_per_px</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.03903357</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>px^-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>field_density_without_flagged_per_px</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.03451624</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>px^-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>field_density_in_roi_per_px</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>px^-1</t>
         </is>
       </c>
     </row>
@@ -932,7 +1424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:W17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -976,6 +1468,81 @@
           <t>mean_edge_length_px</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>perimeter_px</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ring_area_r30_px2</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>ring_area_r60_px2</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>in_frame_fraction_r30</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>in_frame_fraction_r60</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ring_density_r30</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>ring_density_r60</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>roots_per_100px_perimeter</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>ring_attached_length_r30_px</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>ring_attached_length_r60_px</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>ring_length_w_r30_px</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>ring_length_w_r60_px</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>sholl_crossings_r10</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>sholl_crossings_r20</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>sholl_crossings_r30</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1001,6 +1568,51 @@
       </c>
       <c r="H2" t="n">
         <v>31.3028</v>
+      </c>
+      <c r="I2" t="n">
+        <v>215.2315</v>
+      </c>
+      <c r="J2" t="n">
+        <v>5617</v>
+      </c>
+      <c r="K2" t="n">
+        <v>12694</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.6363</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.5983000000000001</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.03133345</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.04064913</v>
+      </c>
+      <c r="P2" t="n">
+        <v>2.7877</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>176</v>
+      </c>
+      <c r="R2" t="n">
+        <v>382</v>
+      </c>
+      <c r="S2" t="n">
+        <v>200.267</v>
+      </c>
+      <c r="T2" t="n">
+        <v>588.3158</v>
+      </c>
+      <c r="U2" t="n">
+        <v>6</v>
+      </c>
+      <c r="V2" t="n">
+        <v>5</v>
+      </c>
+      <c r="W2" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -1028,6 +1640,51 @@
       <c r="H3" t="n">
         <v>33.5078</v>
       </c>
+      <c r="I3" t="n">
+        <v>126.468</v>
+      </c>
+      <c r="J3" t="n">
+        <v>6226</v>
+      </c>
+      <c r="K3" t="n">
+        <v>14794</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.02842917</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.03291875</v>
+      </c>
+      <c r="P3" t="n">
+        <v>3.1629</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>106</v>
+      </c>
+      <c r="R3" t="n">
+        <v>202</v>
+      </c>
+      <c r="S3" t="n">
+        <v>202.8944</v>
+      </c>
+      <c r="T3" t="n">
+        <v>542.3452</v>
+      </c>
+      <c r="U3" t="n">
+        <v>4</v>
+      </c>
+      <c r="V3" t="n">
+        <v>7</v>
+      </c>
+      <c r="W3" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1054,6 +1711,51 @@
       <c r="H4" t="n">
         <v>19.5291</v>
       </c>
+      <c r="I4" t="n">
+        <v>160.6396</v>
+      </c>
+      <c r="J4" t="n">
+        <v>6976</v>
+      </c>
+      <c r="K4" t="n">
+        <v>18799</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.9774</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.03125</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.03255492</v>
+      </c>
+      <c r="P4" t="n">
+        <v>3.1126</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>136</v>
+      </c>
+      <c r="R4" t="n">
+        <v>185</v>
+      </c>
+      <c r="S4" t="n">
+        <v>246.7939</v>
+      </c>
+      <c r="T4" t="n">
+        <v>688.2275</v>
+      </c>
+      <c r="U4" t="n">
+        <v>4</v>
+      </c>
+      <c r="V4" t="n">
+        <v>8</v>
+      </c>
+      <c r="W4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1080,6 +1782,51 @@
       <c r="H5" t="n">
         <v>27.6565</v>
       </c>
+      <c r="I5" t="n">
+        <v>151.7817</v>
+      </c>
+      <c r="J5" t="n">
+        <v>6752</v>
+      </c>
+      <c r="K5" t="n">
+        <v>15321</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.02962085</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.03655114</v>
+      </c>
+      <c r="P5" t="n">
+        <v>3.2942</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>149</v>
+      </c>
+      <c r="R5" t="n">
+        <v>207</v>
+      </c>
+      <c r="S5" t="n">
+        <v>221.9239</v>
+      </c>
+      <c r="T5" t="n">
+        <v>623.3158</v>
+      </c>
+      <c r="U5" t="n">
+        <v>5</v>
+      </c>
+      <c r="V5" t="n">
+        <v>7</v>
+      </c>
+      <c r="W5" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1106,6 +1853,51 @@
       <c r="H6" t="n">
         <v>33.6621</v>
       </c>
+      <c r="I6" t="n">
+        <v>322.0427</v>
+      </c>
+      <c r="J6" t="n">
+        <v>11663</v>
+      </c>
+      <c r="K6" t="n">
+        <v>28685</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.02263569</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.02844692</v>
+      </c>
+      <c r="P6" t="n">
+        <v>2.1736</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>172</v>
+      </c>
+      <c r="R6" t="n">
+        <v>304</v>
+      </c>
+      <c r="S6" t="n">
+        <v>294.3503</v>
+      </c>
+      <c r="T6" t="n">
+        <v>920.193</v>
+      </c>
+      <c r="U6" t="n">
+        <v>8</v>
+      </c>
+      <c r="V6" t="n">
+        <v>11</v>
+      </c>
+      <c r="W6" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1132,6 +1924,51 @@
       <c r="H7" t="n">
         <v>28.4599</v>
       </c>
+      <c r="I7" t="n">
+        <v>438.5168</v>
+      </c>
+      <c r="J7" t="n">
+        <v>13901</v>
+      </c>
+      <c r="K7" t="n">
+        <v>31616</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.04783829</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.04674848</v>
+      </c>
+      <c r="P7" t="n">
+        <v>2.5085</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>532</v>
+      </c>
+      <c r="R7" t="n">
+        <v>1012</v>
+      </c>
+      <c r="S7" t="n">
+        <v>758.3107</v>
+      </c>
+      <c r="T7" t="n">
+        <v>1693.2317</v>
+      </c>
+      <c r="U7" t="n">
+        <v>18</v>
+      </c>
+      <c r="V7" t="n">
+        <v>20</v>
+      </c>
+      <c r="W7" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1158,6 +1995,51 @@
       <c r="H8" t="n">
         <v>36.2452</v>
       </c>
+      <c r="I8" t="n">
+        <v>211.9239</v>
+      </c>
+      <c r="J8" t="n">
+        <v>8845</v>
+      </c>
+      <c r="K8" t="n">
+        <v>21455</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.03448276</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.03388488</v>
+      </c>
+      <c r="P8" t="n">
+        <v>3.7749</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>204</v>
+      </c>
+      <c r="R8" t="n">
+        <v>332</v>
+      </c>
+      <c r="S8" t="n">
+        <v>343.2914</v>
+      </c>
+      <c r="T8" t="n">
+        <v>824.0386999999999</v>
+      </c>
+      <c r="U8" t="n">
+        <v>8</v>
+      </c>
+      <c r="V8" t="n">
+        <v>9</v>
+      </c>
+      <c r="W8" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1184,6 +2066,51 @@
       <c r="H9" t="n">
         <v>20.706</v>
       </c>
+      <c r="I9" t="n">
+        <v>359.1909</v>
+      </c>
+      <c r="J9" t="n">
+        <v>12383</v>
+      </c>
+      <c r="K9" t="n">
+        <v>27034</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.9025</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.02576112</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.02452467</v>
+      </c>
+      <c r="P9" t="n">
+        <v>2.784</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>276</v>
+      </c>
+      <c r="R9" t="n">
+        <v>371</v>
+      </c>
+      <c r="S9" t="n">
+        <v>353.8061</v>
+      </c>
+      <c r="T9" t="n">
+        <v>741.3402</v>
+      </c>
+      <c r="U9" t="n">
+        <v>10</v>
+      </c>
+      <c r="V9" t="n">
+        <v>10</v>
+      </c>
+      <c r="W9" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1210,6 +2137,51 @@
       <c r="H10" t="n">
         <v>35.0728</v>
       </c>
+      <c r="I10" t="n">
+        <v>302.4508</v>
+      </c>
+      <c r="J10" t="n">
+        <v>11295</v>
+      </c>
+      <c r="K10" t="n">
+        <v>27170</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.03461709</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.0354067</v>
+      </c>
+      <c r="P10" t="n">
+        <v>3.3063</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>313</v>
+      </c>
+      <c r="R10" t="n">
+        <v>483</v>
+      </c>
+      <c r="S10" t="n">
+        <v>439.6468</v>
+      </c>
+      <c r="T10" t="n">
+        <v>1078.7615</v>
+      </c>
+      <c r="U10" t="n">
+        <v>13</v>
+      </c>
+      <c r="V10" t="n">
+        <v>15</v>
+      </c>
+      <c r="W10" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1236,6 +2208,51 @@
       <c r="H11" t="n">
         <v>45.9647</v>
       </c>
+      <c r="I11" t="n">
+        <v>309.5219</v>
+      </c>
+      <c r="J11" t="n">
+        <v>11337</v>
+      </c>
+      <c r="K11" t="n">
+        <v>28286</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.03378319</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.03814608</v>
+      </c>
+      <c r="P11" t="n">
+        <v>2.5846</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>309</v>
+      </c>
+      <c r="R11" t="n">
+        <v>705</v>
+      </c>
+      <c r="S11" t="n">
+        <v>433.7473</v>
+      </c>
+      <c r="T11" t="n">
+        <v>1229.7149</v>
+      </c>
+      <c r="U11" t="n">
+        <v>10</v>
+      </c>
+      <c r="V11" t="n">
+        <v>13</v>
+      </c>
+      <c r="W11" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1262,6 +2279,51 @@
       <c r="H12" t="n">
         <v>32.211</v>
       </c>
+      <c r="I12" t="n">
+        <v>468.2742</v>
+      </c>
+      <c r="J12" t="n">
+        <v>15363</v>
+      </c>
+      <c r="K12" t="n">
+        <v>34096</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.03944542</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.04545988</v>
+      </c>
+      <c r="P12" t="n">
+        <v>2.7762</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>480</v>
+      </c>
+      <c r="R12" t="n">
+        <v>1020</v>
+      </c>
+      <c r="S12" t="n">
+        <v>684.9848</v>
+      </c>
+      <c r="T12" t="n">
+        <v>1745.9058</v>
+      </c>
+      <c r="U12" t="n">
+        <v>15</v>
+      </c>
+      <c r="V12" t="n">
+        <v>23</v>
+      </c>
+      <c r="W12" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1288,6 +2350,51 @@
       <c r="H13" t="n">
         <v>22.7438</v>
       </c>
+      <c r="I13" t="n">
+        <v>422.9777</v>
+      </c>
+      <c r="J13" t="n">
+        <v>13165</v>
+      </c>
+      <c r="K13" t="n">
+        <v>30001</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.03410558</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.03603213</v>
+      </c>
+      <c r="P13" t="n">
+        <v>3.0734</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>331</v>
+      </c>
+      <c r="R13" t="n">
+        <v>663</v>
+      </c>
+      <c r="S13" t="n">
+        <v>504.931</v>
+      </c>
+      <c r="T13" t="n">
+        <v>1203.0753</v>
+      </c>
+      <c r="U13" t="n">
+        <v>14</v>
+      </c>
+      <c r="V13" t="n">
+        <v>13</v>
+      </c>
+      <c r="W13" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1313,6 +2420,51 @@
       </c>
       <c r="H14" t="n">
         <v>36.0504</v>
+      </c>
+      <c r="I14" t="n">
+        <v>379.8478</v>
+      </c>
+      <c r="J14" t="n">
+        <v>13296</v>
+      </c>
+      <c r="K14" t="n">
+        <v>32108</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.03542419</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.03242183</v>
+      </c>
+      <c r="P14" t="n">
+        <v>3.4224</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>412</v>
+      </c>
+      <c r="R14" t="n">
+        <v>700</v>
+      </c>
+      <c r="S14" t="n">
+        <v>541.529</v>
+      </c>
+      <c r="T14" t="n">
+        <v>1188.7565</v>
+      </c>
+      <c r="U14" t="n">
+        <v>13</v>
+      </c>
+      <c r="V14" t="n">
+        <v>18</v>
+      </c>
+      <c r="W14" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="15">
@@ -1340,6 +2492,51 @@
       <c r="H15" t="n">
         <v>38.9786</v>
       </c>
+      <c r="I15" t="n">
+        <v>217.9239</v>
+      </c>
+      <c r="J15" t="n">
+        <v>8830</v>
+      </c>
+      <c r="K15" t="n">
+        <v>22986</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.02842582</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.03219351</v>
+      </c>
+      <c r="P15" t="n">
+        <v>2.2944</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>133</v>
+      </c>
+      <c r="R15" t="n">
+        <v>329</v>
+      </c>
+      <c r="S15" t="n">
+        <v>281.2082</v>
+      </c>
+      <c r="T15" t="n">
+        <v>832.524</v>
+      </c>
+      <c r="U15" t="n">
+        <v>5</v>
+      </c>
+      <c r="V15" t="n">
+        <v>9</v>
+      </c>
+      <c r="W15" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1366,6 +2563,51 @@
       <c r="H16" t="n">
         <v>20.2196</v>
       </c>
+      <c r="I16" t="n">
+        <v>332.8944</v>
+      </c>
+      <c r="J16" t="n">
+        <v>10505</v>
+      </c>
+      <c r="K16" t="n">
+        <v>23806</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.8602</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.7919</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.02513089</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.03205074</v>
+      </c>
+      <c r="P16" t="n">
+        <v>1.2016</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>140</v>
+      </c>
+      <c r="R16" t="n">
+        <v>284</v>
+      </c>
+      <c r="S16" t="n">
+        <v>286.0366</v>
+      </c>
+      <c r="T16" t="n">
+        <v>848.5828</v>
+      </c>
+      <c r="U16" t="n">
+        <v>6</v>
+      </c>
+      <c r="V16" t="n">
+        <v>11</v>
+      </c>
+      <c r="W16" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1391,6 +2633,51 @@
       </c>
       <c r="H17" t="n">
         <v>16.1805</v>
+      </c>
+      <c r="I17" t="n">
+        <v>205.7756</v>
+      </c>
+      <c r="J17" t="n">
+        <v>6766</v>
+      </c>
+      <c r="K17" t="n">
+        <v>16357</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.7841</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.714</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.01684895</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.02855047</v>
+      </c>
+      <c r="P17" t="n">
+        <v>1.9439</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>86</v>
+      </c>
+      <c r="R17" t="n">
+        <v>89</v>
+      </c>
+      <c r="S17" t="n">
+        <v>126.8823</v>
+      </c>
+      <c r="T17" t="n">
+        <v>516.9605</v>
+      </c>
+      <c r="U17" t="n">
+        <v>3</v>
+      </c>
+      <c r="V17" t="n">
+        <v>3</v>
+      </c>
+      <c r="W17" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>